<commit_message>
Fix claimed-code migration and fee data
Prevent school code migration from resetting claimed flags on reruns by only creating initial Firestore docs once. Added a one-off repair script to restore legitimately claimed codes that were incorrectly reset by the old migration bug. Also refreshed the fee-related data files and student records to reflect the corrected fee totals.
</commit_message>
<xml_diff>
--- a/2026 - 2027 FEE.xlsx
+++ b/2026 - 2027 FEE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\KBI\ACCOUNTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB1001F-A16E-49DD-B2A1-F42FB38F518D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AC92B81-C2C9-4DC4-9883-CF2DA9C8F58A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1789,7 +1789,7 @@
         <v>4500</v>
       </c>
       <c r="O5" s="24">
-        <v>19560</v>
+        <v>19500</v>
       </c>
       <c r="P5" s="24">
         <v>14330</v>
@@ -1823,14 +1823,14 @@
       </c>
       <c r="Z5" s="24">
         <f t="shared" si="5"/>
-        <v>78390</v>
+        <v>78330</v>
       </c>
       <c r="AA5" s="24">
         <v>0</v>
       </c>
       <c r="AB5" s="20">
         <f t="shared" si="6"/>
-        <v>78390</v>
+        <v>78330</v>
       </c>
       <c r="AC5" s="24" t="str">
         <f t="shared" si="7"/>
@@ -1894,7 +1894,7 @@
         <v>4200</v>
       </c>
       <c r="O6" s="24">
-        <v>19560</v>
+        <v>19500</v>
       </c>
       <c r="P6" s="24">
         <v>14330</v>
@@ -1928,14 +1928,14 @@
       </c>
       <c r="Z6" s="24">
         <f t="shared" si="5"/>
-        <v>67590</v>
+        <v>67530</v>
       </c>
       <c r="AA6" s="24">
         <v>0</v>
       </c>
       <c r="AB6" s="20">
         <f t="shared" si="6"/>
-        <v>67590</v>
+        <v>67530</v>
       </c>
       <c r="AC6" s="24" t="str">
         <f t="shared" si="7"/>
@@ -1999,7 +1999,7 @@
         <v>6000</v>
       </c>
       <c r="O7" s="24">
-        <v>19560</v>
+        <v>19500</v>
       </c>
       <c r="P7" s="24">
         <v>14330</v>
@@ -2033,14 +2033,14 @@
       </c>
       <c r="Z7" s="24">
         <f t="shared" si="5"/>
-        <v>79890</v>
+        <v>79830</v>
       </c>
       <c r="AA7" s="24">
         <v>0</v>
       </c>
       <c r="AB7" s="20">
         <f t="shared" si="6"/>
-        <v>79890</v>
+        <v>79830</v>
       </c>
       <c r="AC7" s="24" t="str">
         <f t="shared" si="7"/>
@@ -2104,7 +2104,7 @@
         <v>6000</v>
       </c>
       <c r="O8" s="24">
-        <v>19560</v>
+        <v>19500</v>
       </c>
       <c r="P8" s="24">
         <v>14330</v>
@@ -2138,14 +2138,14 @@
       </c>
       <c r="Z8" s="24">
         <f t="shared" si="5"/>
-        <v>79890</v>
+        <v>79830</v>
       </c>
       <c r="AA8" s="24">
         <v>0</v>
       </c>
       <c r="AB8" s="20">
         <f t="shared" si="6"/>
-        <v>79890</v>
+        <v>79830</v>
       </c>
       <c r="AC8" s="24" t="str">
         <f t="shared" si="7"/>
@@ -2209,7 +2209,7 @@
         <v>4200</v>
       </c>
       <c r="O9" s="24">
-        <v>19560</v>
+        <v>19500</v>
       </c>
       <c r="P9" s="24">
         <v>14330</v>
@@ -2243,14 +2243,14 @@
       </c>
       <c r="Z9" s="24">
         <f t="shared" si="5"/>
-        <v>67590</v>
+        <v>67530</v>
       </c>
       <c r="AA9" s="24">
         <v>0</v>
       </c>
       <c r="AB9" s="20">
         <f t="shared" si="6"/>
-        <v>67590</v>
+        <v>67530</v>
       </c>
       <c r="AC9" s="24" t="str">
         <f t="shared" si="7"/>
@@ -2314,7 +2314,7 @@
         <v>3000</v>
       </c>
       <c r="O10" s="24">
-        <v>22580</v>
+        <v>22400</v>
       </c>
       <c r="P10" s="24">
         <v>14330</v>
@@ -2348,14 +2348,14 @@
       </c>
       <c r="Z10" s="24">
         <f t="shared" si="5"/>
-        <v>62410</v>
+        <v>62230</v>
       </c>
       <c r="AA10" s="24">
         <v>0</v>
       </c>
       <c r="AB10" s="20">
         <f t="shared" si="6"/>
-        <v>62410</v>
+        <v>62230</v>
       </c>
       <c r="AC10" s="24" t="str">
         <f t="shared" si="7"/>
@@ -2419,7 +2419,7 @@
         <v>3000</v>
       </c>
       <c r="O11" s="24">
-        <v>22580</v>
+        <v>22400</v>
       </c>
       <c r="P11" s="24">
         <v>14330</v>
@@ -2453,14 +2453,14 @@
       </c>
       <c r="Z11" s="24">
         <f t="shared" si="5"/>
-        <v>62410</v>
+        <v>62230</v>
       </c>
       <c r="AA11" s="24">
         <v>0</v>
       </c>
       <c r="AB11" s="20">
         <f t="shared" si="6"/>
-        <v>62410</v>
+        <v>62230</v>
       </c>
       <c r="AC11" s="24" t="str">
         <f t="shared" si="7"/>
@@ -2524,7 +2524,7 @@
         <v>3000</v>
       </c>
       <c r="O12" s="24">
-        <v>22580</v>
+        <v>22400</v>
       </c>
       <c r="P12" s="24">
         <v>14330</v>
@@ -2558,14 +2558,14 @@
       </c>
       <c r="Z12" s="24">
         <f t="shared" si="5"/>
-        <v>70380</v>
+        <v>70200</v>
       </c>
       <c r="AA12" s="24">
         <v>0</v>
       </c>
       <c r="AB12" s="20">
         <f t="shared" si="6"/>
-        <v>70380</v>
+        <v>70200</v>
       </c>
       <c r="AC12" s="24" t="str">
         <f t="shared" si="7"/>
@@ -2629,7 +2629,7 @@
         <v>6000</v>
       </c>
       <c r="O13" s="24">
-        <v>22580</v>
+        <v>22400</v>
       </c>
       <c r="P13" s="24">
         <v>14330</v>
@@ -2663,14 +2663,14 @@
       </c>
       <c r="Z13" s="24">
         <f t="shared" si="5"/>
-        <v>73940</v>
+        <v>73760</v>
       </c>
       <c r="AA13" s="24">
         <v>0</v>
       </c>
       <c r="AB13" s="20">
         <f t="shared" si="6"/>
-        <v>73940</v>
+        <v>73760</v>
       </c>
       <c r="AC13" s="24" t="str">
         <f t="shared" si="7"/>
@@ -2734,7 +2734,7 @@
         <v>3000</v>
       </c>
       <c r="O14" s="24">
-        <v>22580</v>
+        <v>22400</v>
       </c>
       <c r="P14" s="24">
         <v>14330</v>
@@ -2768,14 +2768,14 @@
       </c>
       <c r="Z14" s="24">
         <f t="shared" si="5"/>
-        <v>62890</v>
+        <v>62710</v>
       </c>
       <c r="AA14" s="24">
         <v>0</v>
       </c>
       <c r="AB14" s="20">
         <f t="shared" si="6"/>
-        <v>62890</v>
+        <v>62710</v>
       </c>
       <c r="AC14" s="24" t="str">
         <f t="shared" si="7"/>
@@ -2839,7 +2839,7 @@
         <v>4500</v>
       </c>
       <c r="O15" s="24">
-        <v>22580</v>
+        <v>22400</v>
       </c>
       <c r="P15" s="24">
         <v>14330</v>
@@ -2873,14 +2873,14 @@
       </c>
       <c r="Z15" s="24">
         <f t="shared" si="5"/>
-        <v>72660</v>
+        <v>72480</v>
       </c>
       <c r="AA15" s="24">
         <v>0</v>
       </c>
       <c r="AB15" s="20">
         <f t="shared" si="6"/>
-        <v>72660</v>
+        <v>72480</v>
       </c>
       <c r="AC15" s="24" t="str">
         <f t="shared" si="7"/>
@@ -2944,7 +2944,7 @@
         <v>3000</v>
       </c>
       <c r="O16" s="24">
-        <v>22580</v>
+        <v>22400</v>
       </c>
       <c r="P16" s="24">
         <v>14330</v>
@@ -2978,14 +2978,14 @@
       </c>
       <c r="Z16" s="24">
         <f t="shared" si="5"/>
-        <v>62910</v>
+        <v>62730</v>
       </c>
       <c r="AA16" s="24">
         <v>0</v>
       </c>
       <c r="AB16" s="20">
         <f t="shared" si="6"/>
-        <v>62910</v>
+        <v>62730</v>
       </c>
       <c r="AC16" s="24" t="str">
         <f t="shared" si="7"/>
@@ -3049,7 +3049,7 @@
         <v>3000</v>
       </c>
       <c r="O17" s="24">
-        <v>22580</v>
+        <v>22400</v>
       </c>
       <c r="P17" s="24">
         <v>14330</v>
@@ -3083,14 +3083,14 @@
       </c>
       <c r="Z17" s="24">
         <f t="shared" si="5"/>
-        <v>62410</v>
+        <v>62230</v>
       </c>
       <c r="AA17" s="24">
         <v>0</v>
       </c>
       <c r="AB17" s="20">
         <f t="shared" si="6"/>
-        <v>62410</v>
+        <v>62230</v>
       </c>
       <c r="AC17" s="24" t="str">
         <f t="shared" si="7"/>
@@ -3154,7 +3154,7 @@
         <v>4200</v>
       </c>
       <c r="O18" s="24">
-        <v>22580</v>
+        <v>22400</v>
       </c>
       <c r="P18" s="24">
         <v>14330</v>
@@ -3188,14 +3188,14 @@
       </c>
       <c r="Z18" s="24">
         <f t="shared" si="5"/>
-        <v>70610</v>
+        <v>70430</v>
       </c>
       <c r="AA18" s="24">
         <v>0</v>
       </c>
       <c r="AB18" s="20">
         <f t="shared" si="6"/>
-        <v>70610</v>
+        <v>70430</v>
       </c>
       <c r="AC18" s="24" t="str">
         <f t="shared" si="7"/>
@@ -3259,7 +3259,7 @@
         <v>3000</v>
       </c>
       <c r="O19" s="24">
-        <v>22580</v>
+        <v>22400</v>
       </c>
       <c r="P19" s="24">
         <v>14330</v>
@@ -3293,14 +3293,14 @@
       </c>
       <c r="Z19" s="24">
         <f t="shared" si="5"/>
-        <v>67265</v>
+        <v>67085</v>
       </c>
       <c r="AA19" s="24">
         <v>0</v>
       </c>
       <c r="AB19" s="20">
         <f t="shared" si="6"/>
-        <v>67265</v>
+        <v>67085</v>
       </c>
       <c r="AC19" s="24" t="str">
         <f t="shared" si="7"/>
@@ -3364,7 +3364,7 @@
         <v>4200</v>
       </c>
       <c r="O20" s="24">
-        <v>22580</v>
+        <v>22400</v>
       </c>
       <c r="P20" s="24">
         <v>14330</v>
@@ -3398,14 +3398,14 @@
       </c>
       <c r="Z20" s="24">
         <f t="shared" si="5"/>
-        <v>78610</v>
+        <v>78430</v>
       </c>
       <c r="AA20" s="24">
         <v>0</v>
       </c>
       <c r="AB20" s="20">
         <f t="shared" si="6"/>
-        <v>78610</v>
+        <v>78430</v>
       </c>
       <c r="AC20" s="24" t="str">
         <f t="shared" si="7"/>
@@ -11587,14 +11587,14 @@
         <v>0</v>
       </c>
       <c r="Z98" s="24">
-        <f t="shared" ref="Z98:Z129" si="35">SUM(J98:Y98)</f>
+        <f t="shared" ref="Z98:Z120" si="35">SUM(J98:Y98)</f>
         <v>77120</v>
       </c>
       <c r="AA98" s="24">
         <v>0</v>
       </c>
       <c r="AB98" s="20">
-        <f t="shared" ref="AB98:AB129" si="36">Z98-AA98</f>
+        <f t="shared" ref="AB98:AB120" si="36">Z98-AA98</f>
         <v>77120</v>
       </c>
       <c r="AC98" s="24" t="str">
@@ -13951,7 +13951,7 @@
       </c>
       <c r="Z121" s="27">
         <f t="shared" si="40"/>
-        <v>7251495</v>
+        <v>7249215</v>
       </c>
       <c r="AA121" s="27">
         <f t="shared" si="40"/>
@@ -13959,7 +13959,7 @@
       </c>
       <c r="AB121" s="27">
         <f t="shared" si="40"/>
-        <v>7160495</v>
+        <v>7158215</v>
       </c>
       <c r="AC121" s="27">
         <f t="shared" si="40"/>

</xml_diff>

<commit_message>
Update student fee records
Adjusted payment and fee totals for selected students in the term 1 data, and refreshed the associated fee sheet and parent code mappings used by the school system.
</commit_message>
<xml_diff>
--- a/2026 - 2027 FEE.xlsx
+++ b/2026 - 2027 FEE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\KBI\ACCOUNTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96B6D6AD-C843-43BA-B1C8-0C59B36561F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62977A2E-3E9F-409E-81F8-E82B394EEF21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1ST TERM ACCOUNT" sheetId="14" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="266">
   <si>
     <t>LAST NAME</t>
   </si>
@@ -830,6 +830,12 @@
   <si>
     <t>AKANDE FAMILY</t>
   </si>
+  <si>
+    <t>NIP:paul onyezuoke udenson</t>
+  </si>
+  <si>
+    <t>UDENSON FAMILY</t>
+  </si>
 </sst>
 </file>
 
@@ -13846,11 +13852,11 @@
         <v>36390</v>
       </c>
       <c r="AA118" s="24">
-        <v>0</v>
+        <v>7070</v>
       </c>
       <c r="AB118" s="20">
         <f t="shared" si="36"/>
-        <v>36390</v>
+        <v>29320</v>
       </c>
       <c r="AC118" s="24" t="str">
         <f t="shared" si="37"/>
@@ -13877,7 +13883,7 @@
         <v>30</v>
       </c>
       <c r="D119" s="23">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="E119" s="24">
         <v>0</v>
@@ -13900,7 +13906,7 @@
       </c>
       <c r="K119" s="24">
         <f t="shared" si="31"/>
-        <v>19500</v>
+        <v>18200</v>
       </c>
       <c r="L119" s="24">
         <f t="shared" si="32"/>
@@ -13908,7 +13914,7 @@
       </c>
       <c r="M119" s="24">
         <f t="shared" si="33"/>
-        <v>750</v>
+        <v>700</v>
       </c>
       <c r="N119" s="24">
         <f t="shared" si="34"/>
@@ -13949,14 +13955,14 @@
       </c>
       <c r="Z119" s="24">
         <f t="shared" si="35"/>
-        <v>44280</v>
+        <v>42930</v>
       </c>
       <c r="AA119" s="24">
-        <v>0</v>
+        <v>42930</v>
       </c>
       <c r="AB119" s="20">
         <f t="shared" si="36"/>
-        <v>44280</v>
+        <v>0</v>
       </c>
       <c r="AC119" s="24" t="str">
         <f t="shared" si="37"/>
@@ -13970,7 +13976,9 @@
         <f t="shared" si="39"/>
         <v/>
       </c>
-      <c r="AF119" s="25"/>
+      <c r="AF119" s="25" t="s">
+        <v>259</v>
+      </c>
     </row>
     <row r="120" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A120" s="22" t="s">
@@ -14139,15 +14147,15 @@
       </c>
       <c r="Z121" s="28">
         <f t="shared" si="40"/>
-        <v>7235925</v>
+        <v>7234575</v>
       </c>
       <c r="AA121" s="28">
         <f t="shared" si="40"/>
-        <v>304975</v>
+        <v>354975</v>
       </c>
       <c r="AB121" s="28">
         <f t="shared" si="40"/>
-        <v>6930950</v>
+        <v>6879600</v>
       </c>
       <c r="AC121" s="28">
         <f t="shared" si="40"/>
@@ -22554,6 +22562,23 @@
         <v>263</v>
       </c>
     </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A10" s="8">
+        <v>46266</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>264</v>
+      </c>
+      <c r="D10" s="9">
+        <v>50000</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>265</v>
+      </c>
+    </row>
     <row r="13" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>

</xml_diff>

<commit_message>
Update fee records and parent mappings
Refresh the 2026-2027 fee workbook, parent code sheet, and first-term student ledger with the latest payment and balance data. This update corrects selected student fee totals, paid amounts, and balances to reflect current records and align the parent mapping data with the updated student information.
</commit_message>
<xml_diff>
--- a/2026 - 2027 FEE.xlsx
+++ b/2026 - 2027 FEE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\KBI\ACCOUNTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83457E3A-BDF4-4CB9-AC26-808051A1DBB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12EF9B45-0C21-4664-9312-7EC81E0C373A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1ST TERM ACCOUNT" sheetId="14" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="276">
   <si>
     <t>LAST NAME</t>
   </si>
@@ -839,6 +839,33 @@
   <si>
     <t>ADEDAMOLA IREMIDE</t>
   </si>
+  <si>
+    <t>NIP:SEYI OLOWE</t>
+  </si>
+  <si>
+    <t>ADENIYI SAMUEL</t>
+  </si>
+  <si>
+    <t>AKINWUMI DAVID</t>
+  </si>
+  <si>
+    <t>MONIEPOINT</t>
+  </si>
+  <si>
+    <t>OMOWUNMI AFOLASADE AWOITE</t>
+  </si>
+  <si>
+    <t>FRIDAY OGECHUKWU UKOH</t>
+  </si>
+  <si>
+    <t>PETER FAVOUR</t>
+  </si>
+  <si>
+    <t>EDEM ZENITH</t>
+  </si>
+  <si>
+    <t>DAVID JESUTOFUNMI DARA</t>
+  </si>
 </sst>
 </file>
 
@@ -4058,11 +4085,11 @@
         <v>79830</v>
       </c>
       <c r="AA25" s="24">
-        <v>0</v>
+        <v>60000</v>
       </c>
       <c r="AB25" s="20">
         <f t="shared" si="6"/>
-        <v>79830</v>
+        <v>19830</v>
       </c>
       <c r="AC25" s="24" t="str">
         <f t="shared" si="7"/>
@@ -6490,7 +6517,7 @@
         <v>248</v>
       </c>
       <c r="D48" s="23">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="E48" s="24">
         <v>0</v>
@@ -6513,7 +6540,7 @@
       </c>
       <c r="K48" s="24">
         <f t="shared" si="12"/>
-        <v>28000</v>
+        <v>26600</v>
       </c>
       <c r="L48" s="24">
         <f t="shared" si="13"/>
@@ -6525,7 +6552,7 @@
       </c>
       <c r="N48" s="24">
         <f t="shared" si="15"/>
-        <v>5000</v>
+        <v>4750</v>
       </c>
       <c r="O48" s="24">
         <v>28790</v>
@@ -6562,14 +6589,14 @@
       </c>
       <c r="Z48" s="24">
         <f t="shared" si="16"/>
+        <v>77370</v>
+      </c>
+      <c r="AA48" s="24">
         <v>79020</v>
-      </c>
-      <c r="AA48" s="24">
-        <v>0</v>
       </c>
       <c r="AB48" s="20">
         <f t="shared" si="17"/>
-        <v>79020</v>
+        <v>-1650</v>
       </c>
       <c r="AC48" s="24" t="str">
         <f t="shared" si="7"/>
@@ -6585,7 +6612,7 @@
       </c>
       <c r="AF48" s="25" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>BONUS</v>
       </c>
     </row>
     <row r="49" spans="1:32" x14ac:dyDescent="0.25">
@@ -6674,11 +6701,11 @@
         <v>82800</v>
       </c>
       <c r="AA49" s="24">
-        <v>0</v>
+        <v>42350</v>
       </c>
       <c r="AB49" s="20">
         <f t="shared" si="17"/>
-        <v>82800</v>
+        <v>40450</v>
       </c>
       <c r="AC49" s="24" t="str">
         <f t="shared" si="7"/>
@@ -12011,14 +12038,14 @@
         <v>0</v>
       </c>
       <c r="Z98" s="24">
-        <f t="shared" ref="Z98:Z129" si="34">SUM(J98:Y98)</f>
+        <f t="shared" ref="Z98:Z120" si="34">SUM(J98:Y98)</f>
         <v>57980</v>
       </c>
       <c r="AA98" s="24">
         <v>0</v>
       </c>
       <c r="AB98" s="20">
-        <f t="shared" ref="AB98:AB129" si="35">Z98-AA98</f>
+        <f t="shared" ref="AB98:AB120" si="35">Z98-AA98</f>
         <v>57980</v>
       </c>
       <c r="AC98" s="24" t="str">
@@ -12887,11 +12914,11 @@
         <v>85900</v>
       </c>
       <c r="AA106" s="24">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="AB106" s="20">
         <f t="shared" si="35"/>
-        <v>85900</v>
+        <v>35900</v>
       </c>
       <c r="AC106" s="24" t="str">
         <f t="shared" si="25"/>
@@ -14497,15 +14524,15 @@
       </c>
       <c r="Z121" s="28">
         <f t="shared" si="36"/>
-        <v>7291945</v>
+        <v>7290295</v>
       </c>
       <c r="AA121" s="28">
         <f t="shared" si="36"/>
-        <v>397115</v>
+        <v>628485</v>
       </c>
       <c r="AB121" s="28">
         <f t="shared" si="36"/>
-        <v>6894830</v>
+        <v>6661810</v>
       </c>
       <c r="AC121" s="28">
         <f t="shared" si="36"/>
@@ -22729,10 +22756,10 @@
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="18" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" style="7" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="53.140625" style="7" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35" style="7" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.7109375" style="7" customWidth="1"/>
     <col min="7" max="7" width="4.85546875" style="7" customWidth="1"/>
     <col min="8" max="23" width="24.140625" style="7" customWidth="1"/>
@@ -22946,11 +22973,39 @@
         <v>266</v>
       </c>
     </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A12" s="8">
+        <v>46271</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="D12" s="9">
+        <v>60000</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>268</v>
+      </c>
+    </row>
     <row r="13" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="7"/>
+      <c r="A13" s="8">
+        <v>46270</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="D13" s="9">
+        <v>79020</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>275</v>
+      </c>
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
       <c r="H13" s="7"/>
@@ -22972,10 +23027,21 @@
       <c r="X13" s="7"/>
     </row>
     <row r="14" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="7"/>
+      <c r="A14" s="8">
+        <v>46270</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="D14" s="9">
+        <v>42350</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>274</v>
+      </c>
       <c r="F14" s="7"/>
       <c r="G14" s="7"/>
       <c r="H14" s="7"/>
@@ -22997,10 +23063,21 @@
       <c r="X14" s="7"/>
     </row>
     <row r="15" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="7"/>
+      <c r="A15" s="8">
+        <v>46270</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="D15" s="9">
+        <v>50000</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>273</v>
+      </c>
       <c r="F15" s="7"/>
       <c r="G15" s="7"/>
       <c r="H15" s="7"/>

</xml_diff>

<commit_message>
Refresh fee records and payments
Updated the 2026-2027 fee workbook, parent code mappings, and the first-term student ledger. This includes a corrected payment entry for one student, adjusting total paid and remaining balance in the exported student records.
</commit_message>
<xml_diff>
--- a/2026 - 2027 FEE.xlsx
+++ b/2026 - 2027 FEE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\KBI\ACCOUNTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73B291D2-5646-4D7E-A0FC-35ACFAE817AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36C1F0EF-02A9-49BB-BEC6-09CCEF8DA40E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1ST TERM ACCOUNT" sheetId="14" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="288">
   <si>
     <t>LAST NAME</t>
   </si>
@@ -891,10 +891,16 @@
     <t>JAMIU FAIZAH</t>
   </si>
   <si>
-    <t>IP:KAYODE MATHEW OLUWASEUN-ISRAEL 1ST TERM</t>
+    <t>OLUWASEUN ISRAEL</t>
   </si>
   <si>
-    <t>OLUWASEUN ISRAEL</t>
+    <t>NIP:KAYODE MATHEW OLUWASEUN-ISRAEL 1ST TERM</t>
+  </si>
+  <si>
+    <t>NIP:OLATUNDE BUKOLA ALICE</t>
+  </si>
+  <si>
+    <t>OLATUNDE FAITHFULNESS</t>
   </si>
 </sst>
 </file>
@@ -11087,11 +11093,11 @@
         <v>56930</v>
       </c>
       <c r="AA89" s="24">
-        <v>0</v>
+        <v>24700</v>
       </c>
       <c r="AB89" s="20">
         <f t="shared" si="28"/>
-        <v>56930</v>
+        <v>32230</v>
       </c>
       <c r="AC89" s="24" t="str">
         <f t="shared" si="29"/>
@@ -12064,14 +12070,14 @@
         <v>-10000</v>
       </c>
       <c r="Z98" s="24">
-        <f t="shared" ref="Z98:Z129" si="38">SUM(J98:Y98)</f>
+        <f t="shared" ref="Z98:Z122" si="38">SUM(J98:Y98)</f>
         <v>31790</v>
       </c>
       <c r="AA98" s="24">
         <v>33140</v>
       </c>
       <c r="AB98" s="20">
-        <f t="shared" ref="AB98:AB129" si="39">Z98-AA98</f>
+        <f t="shared" ref="AB98:AB122" si="39">Z98-AA98</f>
         <v>-1350</v>
       </c>
       <c r="AC98" s="24" t="str">
@@ -14775,11 +14781,11 @@
       </c>
       <c r="AA123" s="28">
         <f t="shared" si="44"/>
-        <v>921465</v>
+        <v>946165</v>
       </c>
       <c r="AB123" s="28">
         <f>SUM(AB2:AB122)</f>
-        <v>6577170</v>
+        <v>6552470</v>
       </c>
       <c r="AC123" s="28">
         <f t="shared" ref="AC123:AF123" si="45">SUM(AC2:AC122)</f>
@@ -23007,7 +23013,7 @@
   <cols>
     <col min="1" max="1" width="14" style="8" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="66.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="68.85546875" style="7" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.5703125" style="9" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="35" style="7" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.7109375" style="7" customWidth="1"/>
@@ -23500,13 +23506,13 @@
         <v>250</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D20" s="12">
         <v>33140</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F20" s="7"/>
       <c r="G20" s="7"/>
@@ -23529,10 +23535,21 @@
       <c r="X20" s="7"/>
     </row>
     <row r="21" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="7"/>
+      <c r="A21" s="8">
+        <v>46275</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="D21" s="9">
+        <v>24700</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>287</v>
+      </c>
       <c r="F21" s="7"/>
       <c r="G21" s="7"/>
       <c r="H21" s="7"/>

</xml_diff>